<commit_message>
chore: bump gvsoc_rvvi (parity-audit closure: lanes added, PMP fix, matrix all expected-pass)
Close the audit actions: the two missing sign-off lanes join quick_val
(load_store_rs1_zero PASS; all_csr_por characterized, then root-caused to
the model declaring the PMP CSR bank the RTL does not have and fixed
personality-side), the parity report and the GVSOC test-list matrix record
the closure: 427/427 test points all expected-pass, zero xfail left from
the audit.
</commit_message>
<xml_diff>
--- a/cv32e40p/docs/VerifPlans/Simulation/CV32E40Pv2_test_list_GVSOC.xlsx
+++ b/cv32e40p/docs/VerifPlans/Simulation/CV32E40Pv2_test_list_GVSOC.xlsx
@@ -7047,19 +7047,19 @@
           <t>no changes from v1</t>
         </is>
       </c>
-      <c r="S72" s="113" t="inlineStr">
-        <is>
-          <t>GAP: lane da aggiungere</t>
-        </is>
-      </c>
-      <c r="T72" s="113" t="inlineStr">
-        <is>
-          <t>GAP: lane da aggiungere</t>
-        </is>
-      </c>
-      <c r="U72" s="113" t="inlineStr">
-        <is>
-          <t>GAP: lane da aggiungere</t>
+      <c r="S72" s="110" t="inlineStr">
+        <is>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 2212s - divergenza pmpcfg0 root-caused e fixata (banca PMP undeclared in Cv32e40pCsr, spec-driven)</t>
+        </is>
+      </c>
+      <c r="T72" s="110" t="inlineStr">
+        <is>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 2212s - divergenza pmpcfg0 root-caused e fixata (banca PMP undeclared in Cv32e40pCsr, spec-driven)</t>
+        </is>
+      </c>
+      <c r="U72" s="110" t="inlineStr">
+        <is>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 2212s - divergenza pmpcfg0 root-caused e fixata (banca PMP undeclared in Cv32e40pCsr, spec-driven)</t>
         </is>
       </c>
     </row>
@@ -8667,19 +8667,19 @@
           <t>no changes from v1</t>
         </is>
       </c>
-      <c r="S97" s="113" t="inlineStr">
-        <is>
-          <t>GAP: lane da aggiungere</t>
-        </is>
-      </c>
-      <c r="T97" s="113" t="inlineStr">
-        <is>
-          <t>GAP: lane da aggiungere</t>
-        </is>
-      </c>
-      <c r="U97" s="113" t="inlineStr">
-        <is>
-          <t>GAP: lane da aggiungere</t>
+      <c r="S97" s="110" t="inlineStr">
+        <is>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 28s (parity follow-up)</t>
+        </is>
+      </c>
+      <c r="T97" s="110" t="inlineStr">
+        <is>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 28s (parity follow-up)</t>
+        </is>
+      </c>
+      <c r="U97" s="110" t="inlineStr">
+        <is>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 28s (parity follow-up)</t>
         </is>
       </c>
     </row>
@@ -15019,7 +15019,6 @@
           <t>asse XPULP coperto da varianti dedicate (pulp_* /_xpulp)</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -15057,7 +15056,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu, floating_pt_instr_en)</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -15095,7 +15093,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu_zfinx, floating_pt_zfinx_instr_en)</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -15380,7 +15377,6 @@
           <t>corev_rand_debug_ebreak_xpulp [pulp] PASS</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>debug-trace\CV32E40Pv2_debug</t>
@@ -15628,7 +15624,6 @@
           <t>corev_rand_debug_single_step_xpulp [pulp] PASS</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>debug-trace\CV32E40Pv2_debug</t>
@@ -15750,7 +15745,6 @@
           <t>corev_rand_fp_instr_data_fwd_test [pulp_fpu] PASS</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Zfinx_F_instructions\CV32E40Pv2_F-Zfinx-instructions micro_architecture/CV32E40Pv2_FPU_register_file</t>
@@ -15788,7 +15782,6 @@
           <t>corev_rand_fp_instr_data_fwd_test [pulp_fpu_zfinx] PASS</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Zfinx_F_instructions\CV32E40Pv2_F-Zfinx-instructions micro_architecture/CV32E40Pv2_FPU_register_file</t>
@@ -15826,7 +15819,6 @@
           <t>corev_rand_fp_instr_mlt_cyc_test [pulp_fpu] PASS</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Zfinx_F_instructions\CV32E40Pv2_F-Zfinx-instructions</t>
@@ -15864,7 +15856,6 @@
           <t>corev_rand_fp_instr_mlt_cyc_test [pulp_fpu_zfinx] PASS</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Zfinx_F_instructions\CV32E40Pv2_F-Zfinx-instructions</t>
@@ -15902,7 +15893,6 @@
           <t>corev_rand_fp_instr_sanity_test [pulp_fpu] PASS</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Zfinx_F_instructions\CV32E40Pv2_F-Zfinx-instructions</t>
@@ -15940,7 +15930,6 @@
           <t>corev_rand_fp_instr_sanity_test [pulp_fpu_zfinx] PASS</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Zfinx_F_instructions\CV32E40Pv2_F-Zfinx-instructions</t>
@@ -15978,7 +15967,6 @@
           <t>corev_rand_fp_instr_test [pulp_fpu] PASS</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>Zfinx_F_instructions\CV32E40Pv2_F-Zfinx-instructions</t>
@@ -16016,7 +16004,6 @@
           <t>corev_rand_fp_instr_test [pulp_fpu_zfinx] PASS</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>Zfinx_F_instructions\CV32E40Pv2_F-Zfinx-instructions</t>
@@ -16054,7 +16041,6 @@
           <t>corev_rand_fp_instr_w_special_ops_test [pulp_fpu] PASS</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>Zfinx_F_instructions\CV32E40Pv2_F-Zfinx-instructions</t>
@@ -16092,7 +16078,6 @@
           <t>corev_rand_fp_instr_w_special_ops_test [pulp_fpu_zfinx] PASS</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>Zfinx_F_instructions\CV32E40Pv2_F-Zfinx-instructions</t>
@@ -16130,7 +16115,6 @@
           <t>corev_fp_mstatus_fs_test [pulp_fpu] PASS</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>micro_architecture/CV32E40Pv2_FPU_register_file</t>
@@ -16168,7 +16152,6 @@
           <t>corev_fp_mstatus_fs_test [pulp_fpu_zfinx] PASS</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>micro_architecture/CV32E40Pv2_FPU_register_file</t>
@@ -16547,7 +16530,6 @@
           <t>asse XPULP coperto da varianti dedicate (pulp_* /_xpulp)</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -16585,7 +16567,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu, floating_pt_instr_en)</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -16623,7 +16604,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu_zfinx, floating_pt_zfinx_instr_en)</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -16661,7 +16641,6 @@
           <t>asse XPULP coperto da varianti dedicate (pulp_* /_xpulp)</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -16699,7 +16678,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu, floating_pt_instr_en)</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -16737,7 +16715,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu_zfinx, floating_pt_zfinx_instr_en)</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -16775,7 +16752,6 @@
           <t>asse XPULP coperto da varianti dedicate (pulp_* /_xpulp)</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -16813,7 +16789,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu, floating_pt_instr_en)</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -16851,7 +16826,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu_zfinx, floating_pt_zfinx_instr_en)</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -17645,7 +17619,6 @@
           <t>asse XPULP coperto da varianti dedicate (pulp_* /_xpulp)</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -17683,7 +17656,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu, floating_pt_instr_en)</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -17721,7 +17693,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu_zfinx, floating_pt_zfinx_instr_en)</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -17754,8 +17725,6 @@
           <t>corev_rand_pulp_with_priv_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -17793,7 +17762,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu, floating_pt_instr_en)</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -17831,7 +17799,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu_zfinx, floating_pt_zfinx_instr_en)</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -17864,7 +17831,6 @@
           <t>corev_rand_pulp_hwloop_count_range_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -17986,7 +17952,6 @@
           <t>corev_rand_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -18108,7 +18073,6 @@
           <t>corev_rand_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -18230,7 +18194,6 @@
           <t>corev_rand_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -18352,7 +18315,6 @@
           <t>corev_rand_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -18474,7 +18436,6 @@
           <t>corev_rand_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -18596,7 +18557,6 @@
           <t>corev_rand_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -18718,7 +18678,6 @@
           <t>corev_rand_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -18840,7 +18799,6 @@
           <t>corev_rand_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -18962,7 +18920,6 @@
           <t>corev_rand_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -19084,7 +19041,6 @@
           <t>corev_rand_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -19206,7 +19162,6 @@
           <t>corev_rand_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -19328,7 +19283,6 @@
           <t>corev_rand_pulp_hwloop_exception [pulp] PASS</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -19450,7 +19404,6 @@
           <t>corev_rand_pulp_hwloop_exception [pulp] PASS</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -19572,7 +19525,6 @@
           <t>corev_rand_pulp_hwloop_exception [pulp] PASS</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -19694,7 +19646,6 @@
           <t>corev_rand_pulp_hwloop_exception [pulp] PASS</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -19816,7 +19767,6 @@
           <t>corev_rand_pulp_hwloop_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
           <t>CV32E40Pv2_xpulp-hwloop</t>
@@ -19938,7 +19888,6 @@
           <t>corev_rand_pulp_hwloop_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -20060,7 +20009,6 @@
           <t>corev_rand_pulp_hwloop_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr">
         <is>
           <t>interrupts\CV32E40Pv2_interrupts xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -20182,7 +20130,6 @@
           <t>corev_rand_pulp_hwloop_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr">
         <is>
           <t>CV32E40Pv2_xpulp-hwloop</t>
@@ -20304,7 +20251,6 @@
           <t>corev_rand_pulp_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-bitmanipulations xpulp_instruction_extensions\CV32E40Pv2_xpulp-general-alu xpulp_instruction_extensions\CV32E40Pv2_xpulp-immediate-branching xpulp_instruction_extensions\CV32E40Pv2_xpulp-multiply-accumulate xpulp_instruction_extensions\CV32E40Pv2_xpulp-postinc-loadstore xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -20426,8 +20372,6 @@
           <t>corev_rand_pulp_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G136" t="inlineStr"/>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -20465,7 +20409,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu, floating_pt_instr_en)</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -20503,7 +20446,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu_zfinx, floating_pt_zfinx_instr_en)</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -20536,7 +20478,6 @@
           <t>corev_rand_pulp_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr">
         <is>
           <t>debug-trace\CV32E40Pv2_debug</t>
@@ -20658,7 +20599,6 @@
           <t>corev_rand_pulp_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
           <t>debug-trace\CV32E40Pv2_debug</t>
@@ -20780,7 +20720,6 @@
           <t>corev_rand_pulp_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr">
         <is>
           <t>debug-trace\CV32E40Pv2_debug</t>
@@ -20902,7 +20841,6 @@
           <t>corev_rand_pulp_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
           <t>debug-trace\CV32E40Pv2_debug</t>
@@ -21024,7 +20962,6 @@
           <t>corev_rand_pulp_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
           <t>interrupts\CV32E40Pv2_interrupts xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -21146,7 +21083,6 @@
           <t>corev_rand_pulp_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
           <t>debug-trace\CV32E40Pv2_debug</t>
@@ -21268,8 +21204,6 @@
           <t>corev_rand_pulp_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G157" t="inlineStr"/>
-      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -21307,7 +21241,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu, floating_pt_instr_en)</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -21345,7 +21278,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu_zfinx, floating_pt_zfinx_instr_en)</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -22638,7 +22570,6 @@
           <t>corev_rand_pulp_mac_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr">
         <is>
           <t>CV32E40Pv2_xpulp-multiply-accumulate</t>
@@ -22760,7 +22691,6 @@
           <t>corev_rand_pulp_simd_instr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G193" t="inlineStr"/>
       <c r="H193" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -22874,15 +22804,14 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>D-ASSENTE</t>
+          <t>A-lane-aggiunta-fix-PMP-20260812</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G196" t="inlineStr"/>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 2212s - divergenza pmpcfg0 root-caused e fixata (banca PMP undeclared in Cv32e40pCsr, spec-driven)</t>
+        </is>
+      </c>
       <c r="H196" t="inlineStr">
         <is>
           <t>priviledged_spec\CV32E40Pv2 - CSR_vplan.md</t>
@@ -22912,15 +22841,14 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>D-ASSENTE</t>
+          <t>A-lane-aggiunta-fix-PMP-20260812</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G197" t="inlineStr"/>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 2212s - divergenza pmpcfg0 root-caused e fixata (banca PMP undeclared in Cv32e40pCsr, spec-driven)</t>
+        </is>
+      </c>
       <c r="H197" t="inlineStr">
         <is>
           <t>priviledged_spec\CV32E40Pv2 - CSR_vplan.md</t>
@@ -22950,15 +22878,14 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>D-ASSENTE</t>
+          <t>A-lane-aggiunta-fix-PMP-20260812</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G198" t="inlineStr"/>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 2212s - divergenza pmpcfg0 root-caused e fixata (banca PMP undeclared in Cv32e40pCsr, spec-driven)</t>
+        </is>
+      </c>
       <c r="H198" t="inlineStr">
         <is>
           <t>priviledged_spec\CV32E40Pv2 - CSR_vplan.md</t>
@@ -23001,7 +22928,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -23039,7 +22965,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -23077,7 +23002,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -23115,7 +23039,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -23153,7 +23076,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -23191,7 +23113,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -23476,7 +23397,6 @@
           <t>cv32e40p_csr_access_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G211" t="inlineStr"/>
       <c r="H211" t="inlineStr">
         <is>
           <t>priviledged_spec\CV32E40Pv2 - CSR_vplan.md</t>
@@ -23724,7 +23644,6 @@
           <t>cv32e40pv2_illegal_ro_csr_access_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G217" t="inlineStr"/>
       <c r="H217" t="inlineStr">
         <is>
           <t>priviledged_spec\CV32E40Pv2 - CSR_vplan.md</t>
@@ -24481,7 +24400,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -24519,7 +24437,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -24557,7 +24474,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -24595,7 +24511,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -24633,7 +24548,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -24671,7 +24585,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -24704,8 +24617,6 @@
           <t>fpu_bugs_test [pulp_fpu] PASS</t>
         </is>
       </c>
-      <c r="G241" t="inlineStr"/>
-      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -24738,8 +24649,6 @@
           <t>fpu_bugs_test [pulp_fpu_zfinx] PASS</t>
         </is>
       </c>
-      <c r="G242" t="inlineStr"/>
-      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -24777,7 +24686,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -24815,7 +24723,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -24853,7 +24760,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -24891,7 +24797,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -24929,7 +24834,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -24967,7 +24871,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -25005,7 +24908,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -25043,7 +24945,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -25081,7 +24982,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -25119,7 +25019,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -25157,7 +25056,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -25195,7 +25093,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -25233,7 +25130,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -25271,7 +25167,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -25309,7 +25204,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -25347,7 +25241,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -25385,7 +25278,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -25423,7 +25315,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -25713,7 +25604,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -25751,7 +25641,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -25789,7 +25678,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -25814,16 +25702,14 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>D-ASSENTE</t>
+          <t>A-lane-aggiunta-20260812</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G270" t="inlineStr"/>
-      <c r="H270" t="inlineStr"/>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 28s (parity follow-up)</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -25848,16 +25734,14 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>D-ASSENTE</t>
+          <t>A-lane-aggiunta-20260812</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G271" t="inlineStr"/>
-      <c r="H271" t="inlineStr"/>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 28s (parity follow-up)</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -25882,16 +25766,14 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>D-ASSENTE</t>
+          <t>A-lane-aggiunta-20260812</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G272" t="inlineStr"/>
-      <c r="H272" t="inlineStr"/>
+          <t>A: lane aggiunta 2026-08-12 [pulp] PASS 28s (parity follow-up)</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -25924,8 +25806,6 @@
           <t>matmul_32b_float [pulp_fpu] PASS</t>
         </is>
       </c>
-      <c r="G273" t="inlineStr"/>
-      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -25963,7 +25843,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -26001,7 +25880,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -26039,7 +25917,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -26077,7 +25954,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -26115,7 +25991,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -26153,7 +26028,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -26191,7 +26065,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -26355,7 +26228,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -26393,7 +26265,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -26431,7 +26302,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -26464,7 +26334,6 @@
           <t>pulp_bit_manipulation [pulp] PASS</t>
         </is>
       </c>
-      <c r="G287" t="inlineStr"/>
       <c r="H287" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-bitmanipulations</t>
@@ -26586,7 +26455,6 @@
           <t>pulp_general_alu [pulp] PASS</t>
         </is>
       </c>
-      <c r="G290" t="inlineStr"/>
       <c r="H290" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-general-alu</t>
@@ -26708,7 +26576,6 @@
           <t>pulp_hardware_loop [pulp] PASS</t>
         </is>
       </c>
-      <c r="G293" t="inlineStr"/>
       <c r="H293" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -26830,7 +26697,6 @@
           <t>pulp_hardware_loop_debug_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G296" t="inlineStr"/>
       <c r="H296" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -26952,7 +26818,6 @@
           <t>pulp_hardware_loop_interrupt_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G299" t="inlineStr"/>
       <c r="H299" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -27074,7 +26939,6 @@
           <t>pulp_immediate_branching [pulp] PASS</t>
         </is>
       </c>
-      <c r="G302" t="inlineStr"/>
       <c r="H302" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-immediate-branching</t>
@@ -27196,7 +27060,6 @@
           <t>pulp_multiply_accumulate [pulp] PASS</t>
         </is>
       </c>
-      <c r="G305" t="inlineStr"/>
       <c r="H305" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-multiply-accumulate</t>
@@ -27318,7 +27181,6 @@
           <t>pulp_post_increment_load_store [pulp] PASS</t>
         </is>
       </c>
-      <c r="G308" t="inlineStr"/>
       <c r="H308" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-postinc-loadstore</t>
@@ -27440,7 +27302,6 @@
           <t>pulp_vectorial_add_sub [pulp] PASS</t>
         </is>
       </c>
-      <c r="G311" t="inlineStr"/>
       <c r="H311" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -27562,7 +27423,6 @@
           <t>pulp_vectorial_avg [pulp] PASS</t>
         </is>
       </c>
-      <c r="G314" t="inlineStr"/>
       <c r="H314" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -27684,7 +27544,6 @@
           <t>pulp_vectorial_bit_manip [pulp] PASS</t>
         </is>
       </c>
-      <c r="G317" t="inlineStr"/>
       <c r="H317" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -27806,7 +27665,6 @@
           <t>pulp_vectorial_bitwise [pulp] PASS</t>
         </is>
       </c>
-      <c r="G320" t="inlineStr"/>
       <c r="H320" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -27928,7 +27786,6 @@
           <t>pulp_vectorial_comparison_1 [pulp] PASS</t>
         </is>
       </c>
-      <c r="G323" t="inlineStr"/>
       <c r="H323" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -28050,7 +27907,6 @@
           <t>pulp_vectorial_comparison_2 [pulp] PASS</t>
         </is>
       </c>
-      <c r="G326" t="inlineStr"/>
       <c r="H326" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -28172,7 +28028,6 @@
           <t>pulp_vectorial_comparison_3 [pulp] PASS</t>
         </is>
       </c>
-      <c r="G329" t="inlineStr"/>
       <c r="H329" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -28294,7 +28149,6 @@
           <t>pulp_vectorial_complex [pulp] PASS</t>
         </is>
       </c>
-      <c r="G332" t="inlineStr"/>
       <c r="H332" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -28416,7 +28270,6 @@
           <t>pulp_vectorial_dot_product_1 [pulp] PASS</t>
         </is>
       </c>
-      <c r="G335" t="inlineStr"/>
       <c r="H335" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -28538,7 +28391,6 @@
           <t>pulp_vectorial_dot_product_2 [pulp] PASS</t>
         </is>
       </c>
-      <c r="G338" t="inlineStr"/>
       <c r="H338" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -28660,7 +28512,6 @@
           <t>pulp_vectorial_max [pulp] PASS</t>
         </is>
       </c>
-      <c r="G341" t="inlineStr"/>
       <c r="H341" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -28782,7 +28633,6 @@
           <t>pulp_vectorial_min [pulp] PASS</t>
         </is>
       </c>
-      <c r="G344" t="inlineStr"/>
       <c r="H344" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -28904,7 +28754,6 @@
           <t>pulp_vectorial_shift [pulp] PASS</t>
         </is>
       </c>
-      <c r="G347" t="inlineStr"/>
       <c r="H347" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -29026,7 +28875,6 @@
           <t>pulp_vectorial_shuffle_pack [pulp] PASS</t>
         </is>
       </c>
-      <c r="G350" t="inlineStr"/>
       <c r="H350" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-packed-simd</t>
@@ -29279,7 +29127,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -29317,7 +29164,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -29355,7 +29201,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -29393,7 +29238,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -29431,7 +29275,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -29469,7 +29312,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -29507,7 +29349,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -29545,7 +29386,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -29583,7 +29423,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -29616,8 +29455,6 @@
           <t>custom_opcode_illegal_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G365" t="inlineStr"/>
-      <c r="H365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -29655,7 +29492,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -29693,7 +29529,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -29726,8 +29561,6 @@
           <t>debug_hwloop_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G368" t="inlineStr"/>
-      <c r="H368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -29765,7 +29598,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -29803,7 +29635,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -29836,8 +29667,6 @@
           <t>illegal_fp_instr_test [pulp_fpu] PASS</t>
         </is>
       </c>
-      <c r="G371" t="inlineStr"/>
-      <c r="H371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -29870,8 +29699,6 @@
           <t>illegal_fp_instr_test [pulp_fpu_zfinx] PASS</t>
         </is>
       </c>
-      <c r="G372" t="inlineStr"/>
-      <c r="H372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -29904,7 +29731,6 @@
           <t>fpu_func_cov_improve_test [pulp_fpu] PASS</t>
         </is>
       </c>
-      <c r="G373" t="inlineStr"/>
       <c r="H373" t="inlineStr">
         <is>
           <t>micro_architecture/CV32E40Pv2_FPU_register_file</t>
@@ -29942,7 +29768,6 @@
           <t>zfinx_func_cov_improve_test [pulp_fpu_zfinx] PASS</t>
         </is>
       </c>
-      <c r="G374" t="inlineStr"/>
       <c r="H374" t="inlineStr">
         <is>
           <t>micro_architecture/CV32E40Pv2_FPU_register_file</t>
@@ -29980,8 +29805,6 @@
           <t>jalr_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G375" t="inlineStr"/>
-      <c r="H375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -30019,7 +29842,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -30057,7 +29879,6 @@
           <t>programma identico, config non ISS-distinta per questo binario</t>
         </is>
       </c>
-      <c r="H377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -30090,7 +29911,6 @@
           <t>corev_directed_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G378" t="inlineStr"/>
       <c r="H378" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -30212,7 +30032,6 @@
           <t>corev_directed_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G381" t="inlineStr"/>
       <c r="H381" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -30334,7 +30153,6 @@
           <t>corev_directed_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G384" t="inlineStr"/>
       <c r="H384" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -30456,8 +30274,6 @@
           <t>corev_directed_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G387" t="inlineStr"/>
-      <c r="H387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -30495,7 +30311,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu, floating_pt_instr_en)</t>
         </is>
       </c>
-      <c r="H388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -30533,7 +30348,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu_zfinx, floating_pt_zfinx_instr_en)</t>
         </is>
       </c>
-      <c r="H389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -30566,7 +30380,6 @@
           <t>corev_directed_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G390" t="inlineStr"/>
       <c r="H390" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -30688,7 +30501,6 @@
           <t>corev_directed_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G393" t="inlineStr"/>
       <c r="H393" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -30810,7 +30622,6 @@
           <t>corev_directed_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G396" t="inlineStr"/>
       <c r="H396" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -31184,7 +30995,6 @@
           <t>corev_rand_pulp_hwloop_in_debug_rom [pulp] PASS</t>
         </is>
       </c>
-      <c r="G405" t="inlineStr"/>
       <c r="H405" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -31306,7 +31116,6 @@
           <t>corev_directed_for_interrupt_covg_test [pulp_fpu] PASS</t>
         </is>
       </c>
-      <c r="G408" t="inlineStr"/>
       <c r="H408" t="inlineStr">
         <is>
           <t>interrupts\CV32E40Pv2_interrupts</t>
@@ -31386,7 +31195,6 @@
           <t>corev_directed_for_hwloop_covg_test [pulp] PASS</t>
         </is>
       </c>
-      <c r="G410" t="inlineStr"/>
       <c r="H410" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -31513,7 +31321,6 @@
           <t>ufficiale tcfg=floating_pt_instr_en,gen_rand_int</t>
         </is>
       </c>
-      <c r="H413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -31551,7 +31358,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu_zfinx, floating_pt_zfinx_instr_en)</t>
         </is>
       </c>
-      <c r="H414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -31589,7 +31395,6 @@
           <t>ufficiale tcfg=floating_pt_instr_en,gen_rand_int</t>
         </is>
       </c>
-      <c r="H415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -31627,7 +31432,6 @@
           <t>asse FP-random coperto da corev_rand_fp_instr_test (pulp_fpu_zfinx, floating_pt_zfinx_instr_en)</t>
         </is>
       </c>
-      <c r="H416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -31660,7 +31464,6 @@
           <t>corev_directed_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G417" t="inlineStr"/>
       <c r="H417" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -31782,7 +31585,6 @@
           <t>corev_directed_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G420" t="inlineStr"/>
       <c r="H420" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -31904,7 +31706,6 @@
           <t>corev_directed_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G423" t="inlineStr"/>
       <c r="H423" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>
@@ -32026,7 +31827,6 @@
           <t>corev_directed_pulp_hwloop_debug [pulp] PASS</t>
         </is>
       </c>
-      <c r="G426" t="inlineStr"/>
       <c r="H426" t="inlineStr">
         <is>
           <t>xpulp_instruction_extensions\CV32E40Pv2_xpulp-hwloop</t>

</xml_diff>